<commit_message>
M6.1: finance ingestion repo half + finance tab standardization (D-052)
- automation/finance/scrape.js (ported off attic Render/Drive; local CSV; bank_creds.json; israeli-bank-scrapers 6.7.3) + package(-lock).json
- automation/finance_ingest.py: CSV -> lib/sheet (append Finance-Transactions, upsert Finance-Accounts); dedup, fail-loud, seed-safe
- lib/sheet.upsert_rows; tab rename Finance-Budget/Finance-Accounts/Finance-Transactions (config, weekly_briefing, seed + SUMIFS refs, SPEC 6.4/12.2)
- family-finance.{service,timer} + provision (npm ci/creds/timer) + bank_creds.example.json
- 325 tests green (+13 test_finance)
</commit_message>
<xml_diff>
--- a/Family_OS.xlsx
+++ b/Family_OS.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="People" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Calendars" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Calendar-Events" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Reminders" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Finance-Accts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Finance-Txns" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Finance-Bdgt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Goals" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Education" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Health" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Car" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Contacts" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Contracts" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Lists" sheetId="15" state="hidden" r:id="rId15"/>
-    <sheet name="Settings" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="WhatsApp_Inbox" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="WhatsApp_Archive" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendars" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar-Events" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reminders" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance-Accounts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance-Budget" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goals" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Education" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Car" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="14" state="hidden" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhatsApp_Inbox" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhatsApp_Archive" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance-Transactions" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -969,48 +969,47 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="12" customWidth="1" style="27" min="1" max="1"/>
-    <col width="22" customWidth="1" style="27" min="2" max="2"/>
-    <col width="16" customWidth="1" style="27" min="3" max="3"/>
-    <col width="18" customWidth="1" style="27" min="4" max="4"/>
-    <col width="14" customWidth="1" style="27" min="5" max="5"/>
-    <col width="18" customWidth="1" style="27" min="6" max="6"/>
-    <col width="28" customWidth="1" style="27" min="7" max="8"/>
+    <col width="14" customWidth="1" style="27" min="1" max="1"/>
+    <col width="26" customWidth="1" style="27" min="2" max="2"/>
+    <col width="18" customWidth="1" style="27" min="3" max="3"/>
+    <col width="12" customWidth="1" style="27" min="4" max="6"/>
+    <col width="28" customWidth="1" style="27" min="7" max="7"/>
+    <col width="18" customWidth="1" style="27" min="8" max="8"/>
     <col width="24" customWidth="1" style="27" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="28">
       <c r="A1" s="34" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>Person</t>
         </is>
       </c>
       <c r="B1" s="34" t="inlineStr">
         <is>
-          <t>Institution</t>
+          <t>Provider</t>
         </is>
       </c>
       <c r="C1" s="34" t="inlineStr">
         <is>
-          <t>Year/Grade</t>
+          <t>Specialty</t>
         </is>
       </c>
       <c r="D1" s="34" t="inlineStr">
         <is>
-          <t>Teacher/Caregiver</t>
+          <t>Last Visit</t>
         </is>
       </c>
       <c r="E1" s="34" t="inlineStr">
         <is>
-          <t>Next Key Date</t>
+          <t>Next Due</t>
         </is>
       </c>
       <c r="F1" s="34" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Frequency</t>
         </is>
       </c>
       <c r="G1" s="34" t="inlineStr">
@@ -1032,40 +1031,38 @@
     <row r="2" ht="36" customHeight="1" s="28">
       <c r="A2" s="35" t="inlineStr">
         <is>
-          <t>[Child 1]</t>
+          <t>[Adar]</t>
         </is>
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>[Preschool name]</t>
+          <t>Dr. Cohen — Clalit</t>
         </is>
       </c>
       <c r="C2" s="35" t="inlineStr">
         <is>
-          <t>Gan Trom-Hova</t>
-        </is>
-      </c>
-      <c r="D2" s="35" t="inlineStr">
-        <is>
-          <t>[Teacher]</t>
-        </is>
+          <t>Family doctor</t>
+        </is>
+      </c>
+      <c r="D2" s="36" t="n">
+        <v>46032</v>
       </c>
       <c r="E2" s="36" t="n">
-        <v>46266</v>
+        <v>46397</v>
       </c>
       <c r="F2" s="35" t="inlineStr">
         <is>
-          <t>School year start</t>
+          <t>Yearly</t>
         </is>
       </c>
       <c r="G2" s="35" t="inlineStr">
         <is>
-          <t>Buy supplies, label clothes</t>
+          <t>Schedule annual check</t>
         </is>
       </c>
       <c r="H2" s="35" t="inlineStr">
         <is>
-          <t>[teacher@school]</t>
+          <t>[clinic phone]</t>
         </is>
       </c>
       <c r="I2" s="35" t="n"/>
@@ -1073,40 +1070,38 @@
     <row r="3" ht="36" customHeight="1" s="28">
       <c r="A3" s="35" t="inlineStr">
         <is>
-          <t>[Child 1]</t>
+          <t>[Adar]</t>
         </is>
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
-          <t>[Preschool name]</t>
+          <t>Dr. Stern</t>
         </is>
       </c>
       <c r="C3" s="35" t="inlineStr">
         <is>
-          <t>Gan Trom-Hova</t>
-        </is>
-      </c>
-      <c r="D3" s="35" t="inlineStr">
-        <is>
-          <t>[Teacher]</t>
-        </is>
+          <t>Dentist</t>
+        </is>
+      </c>
+      <c r="D3" s="36" t="n">
+        <v>46068</v>
       </c>
       <c r="E3" s="36" t="n">
-        <v>46346</v>
+        <v>46249</v>
       </c>
       <c r="F3" s="35" t="inlineStr">
         <is>
-          <t>Parent-teacher</t>
+          <t>6-month</t>
         </is>
       </c>
       <c r="G3" s="35" t="inlineStr">
         <is>
-          <t>Schedule meeting slot</t>
+          <t>Schedule cleaning</t>
         </is>
       </c>
       <c r="H3" s="35" t="inlineStr">
         <is>
-          <t>[teacher@school]</t>
+          <t>[clinic phone]</t>
         </is>
       </c>
       <c r="I3" s="35" t="n"/>
@@ -1114,80 +1109,154 @@
     <row r="4" ht="36" customHeight="1" s="28">
       <c r="A4" s="35" t="inlineStr">
         <is>
+          <t>[Partner]</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Dr. Levi — Maccabi</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Family doctor</t>
+        </is>
+      </c>
+      <c r="D4" s="36" t="n">
+        <v>45966</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>46331</v>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>Yearly</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="n"/>
+      <c r="H4" s="35" t="inlineStr">
+        <is>
+          <t>[clinic phone]</t>
+        </is>
+      </c>
+      <c r="I4" s="35" t="n"/>
+    </row>
+    <row r="5" ht="36" customHeight="1" s="28">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>[Child 1]</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>Dr. Cohen — Clalit</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>Pediatrician</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>46101</v>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>46285</v>
+      </c>
+      <c r="F5" s="35" t="inlineStr">
+        <is>
+          <t>6-month</t>
+        </is>
+      </c>
+      <c r="G5" s="35" t="inlineStr">
+        <is>
+          <t>Routine check</t>
+        </is>
+      </c>
+      <c r="H5" s="35" t="inlineStr">
+        <is>
+          <t>[clinic phone]</t>
+        </is>
+      </c>
+      <c r="I5" s="35" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1" s="28">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>[Child 1]</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Tipat Halav</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Vaccines</t>
+        </is>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>46113</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>Per schedule</t>
+        </is>
+      </c>
+      <c r="G6" s="35" t="inlineStr">
+        <is>
+          <t>MMR booster</t>
+        </is>
+      </c>
+      <c r="H6" s="35" t="inlineStr">
+        <is>
+          <t>[Tipat Halav phone]</t>
+        </is>
+      </c>
+      <c r="I6" s="35" t="n"/>
+    </row>
+    <row r="7" ht="36" customHeight="1" s="28">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
           <t>[Child 2]</t>
         </is>
       </c>
-      <c r="B4" s="35" t="inlineStr">
-        <is>
-          <t>[Daycare name]</t>
-        </is>
-      </c>
-      <c r="C4" s="35" t="inlineStr">
-        <is>
-          <t>Maon</t>
-        </is>
-      </c>
-      <c r="D4" s="35" t="inlineStr">
-        <is>
-          <t>[Caregiver]</t>
-        </is>
-      </c>
-      <c r="E4" s="36" t="n">
-        <v>46371</v>
-      </c>
-      <c r="F4" s="35" t="inlineStr">
-        <is>
-          <t>1st-grade registration opens</t>
-        </is>
-      </c>
-      <c r="G4" s="35" t="inlineStr">
-        <is>
-          <t>Register on city portal</t>
-        </is>
-      </c>
-      <c r="H4" s="35" t="inlineStr">
-        <is>
-          <t>[city helpdesk]</t>
-        </is>
-      </c>
-      <c r="I4" s="35" t="inlineStr">
-        <is>
-          <t>Adar to lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="28">
-      <c r="A5" s="37" t="n"/>
-      <c r="B5" s="37" t="n"/>
-      <c r="C5" s="37" t="n"/>
-      <c r="D5" s="37" t="n"/>
-      <c r="E5" s="37" t="n"/>
-      <c r="F5" s="37" t="n"/>
-      <c r="G5" s="37" t="n"/>
-      <c r="H5" s="37" t="n"/>
-      <c r="I5" s="37" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="28">
-      <c r="A6" s="37" t="n"/>
-      <c r="B6" s="37" t="n"/>
-      <c r="C6" s="37" t="n"/>
-      <c r="D6" s="37" t="n"/>
-      <c r="E6" s="37" t="n"/>
-      <c r="F6" s="37" t="n"/>
-      <c r="G6" s="37" t="n"/>
-      <c r="H6" s="37" t="n"/>
-      <c r="I6" s="37" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="28">
-      <c r="A7" s="37" t="n"/>
-      <c r="B7" s="37" t="n"/>
-      <c r="C7" s="37" t="n"/>
-      <c r="D7" s="37" t="n"/>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="37" t="n"/>
-      <c r="G7" s="37" t="n"/>
-      <c r="H7" s="37" t="n"/>
-      <c r="I7" s="37" t="n"/>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Tipat Halav</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>Vaccines</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="n">
+        <v>46063</v>
+      </c>
+      <c r="E7" s="36" t="n">
+        <v>46244</v>
+      </c>
+      <c r="F7" s="35" t="inlineStr">
+        <is>
+          <t>Per schedule</t>
+        </is>
+      </c>
+      <c r="G7" s="35" t="inlineStr">
+        <is>
+          <t>12-month vaccines</t>
+        </is>
+      </c>
+      <c r="H7" s="35" t="inlineStr">
+        <is>
+          <t>[Tipat Halav phone]</t>
+        </is>
+      </c>
+      <c r="I7" s="35" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="28">
       <c r="A8" s="37" t="n"/>
@@ -1320,6 +1389,39 @@
       <c r="G19" s="37" t="n"/>
       <c r="H19" s="37" t="n"/>
       <c r="I19" s="37" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="28">
+      <c r="A20" s="37" t="n"/>
+      <c r="B20" s="37" t="n"/>
+      <c r="C20" s="37" t="n"/>
+      <c r="D20" s="37" t="n"/>
+      <c r="E20" s="37" t="n"/>
+      <c r="F20" s="37" t="n"/>
+      <c r="G20" s="37" t="n"/>
+      <c r="H20" s="37" t="n"/>
+      <c r="I20" s="37" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="28">
+      <c r="A21" s="37" t="n"/>
+      <c r="B21" s="37" t="n"/>
+      <c r="C21" s="37" t="n"/>
+      <c r="D21" s="37" t="n"/>
+      <c r="E21" s="37" t="n"/>
+      <c r="F21" s="37" t="n"/>
+      <c r="G21" s="37" t="n"/>
+      <c r="H21" s="37" t="n"/>
+      <c r="I21" s="37" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="28">
+      <c r="A22" s="37" t="n"/>
+      <c r="B22" s="37" t="n"/>
+      <c r="C22" s="37" t="n"/>
+      <c r="D22" s="37" t="n"/>
+      <c r="E22" s="37" t="n"/>
+      <c r="F22" s="37" t="n"/>
+      <c r="G22" s="37" t="n"/>
+      <c r="H22" s="37" t="n"/>
+      <c r="I22" s="37" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E1000">
@@ -1337,481 +1439,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="14" customWidth="1" style="27" min="1" max="1"/>
-    <col width="26" customWidth="1" style="27" min="2" max="2"/>
-    <col width="18" customWidth="1" style="27" min="3" max="3"/>
-    <col width="12" customWidth="1" style="27" min="4" max="6"/>
-    <col width="28" customWidth="1" style="27" min="7" max="7"/>
-    <col width="18" customWidth="1" style="27" min="8" max="8"/>
-    <col width="24" customWidth="1" style="27" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="27.75" customHeight="1" s="28">
-      <c r="A1" s="34" t="inlineStr">
-        <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="B1" s="34" t="inlineStr">
-        <is>
-          <t>Provider</t>
-        </is>
-      </c>
-      <c r="C1" s="34" t="inlineStr">
-        <is>
-          <t>Specialty</t>
-        </is>
-      </c>
-      <c r="D1" s="34" t="inlineStr">
-        <is>
-          <t>Last Visit</t>
-        </is>
-      </c>
-      <c r="E1" s="34" t="inlineStr">
-        <is>
-          <t>Next Due</t>
-        </is>
-      </c>
-      <c r="F1" s="34" t="inlineStr">
-        <is>
-          <t>Frequency</t>
-        </is>
-      </c>
-      <c r="G1" s="34" t="inlineStr">
-        <is>
-          <t>Action Needed</t>
-        </is>
-      </c>
-      <c r="H1" s="34" t="inlineStr">
-        <is>
-          <t>Contact</t>
-        </is>
-      </c>
-      <c r="I1" s="34" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1" s="28">
-      <c r="A2" s="35" t="inlineStr">
-        <is>
-          <t>[Adar]</t>
-        </is>
-      </c>
-      <c r="B2" s="35" t="inlineStr">
-        <is>
-          <t>Dr. Cohen — Clalit</t>
-        </is>
-      </c>
-      <c r="C2" s="35" t="inlineStr">
-        <is>
-          <t>Family doctor</t>
-        </is>
-      </c>
-      <c r="D2" s="36" t="n">
-        <v>46032</v>
-      </c>
-      <c r="E2" s="36" t="n">
-        <v>46397</v>
-      </c>
-      <c r="F2" s="35" t="inlineStr">
-        <is>
-          <t>Yearly</t>
-        </is>
-      </c>
-      <c r="G2" s="35" t="inlineStr">
-        <is>
-          <t>Schedule annual check</t>
-        </is>
-      </c>
-      <c r="H2" s="35" t="inlineStr">
-        <is>
-          <t>[clinic phone]</t>
-        </is>
-      </c>
-      <c r="I2" s="35" t="n"/>
-    </row>
-    <row r="3" ht="36" customHeight="1" s="28">
-      <c r="A3" s="35" t="inlineStr">
-        <is>
-          <t>[Adar]</t>
-        </is>
-      </c>
-      <c r="B3" s="35" t="inlineStr">
-        <is>
-          <t>Dr. Stern</t>
-        </is>
-      </c>
-      <c r="C3" s="35" t="inlineStr">
-        <is>
-          <t>Dentist</t>
-        </is>
-      </c>
-      <c r="D3" s="36" t="n">
-        <v>46068</v>
-      </c>
-      <c r="E3" s="36" t="n">
-        <v>46249</v>
-      </c>
-      <c r="F3" s="35" t="inlineStr">
-        <is>
-          <t>6-month</t>
-        </is>
-      </c>
-      <c r="G3" s="35" t="inlineStr">
-        <is>
-          <t>Schedule cleaning</t>
-        </is>
-      </c>
-      <c r="H3" s="35" t="inlineStr">
-        <is>
-          <t>[clinic phone]</t>
-        </is>
-      </c>
-      <c r="I3" s="35" t="n"/>
-    </row>
-    <row r="4" ht="36" customHeight="1" s="28">
-      <c r="A4" s="35" t="inlineStr">
-        <is>
-          <t>[Partner]</t>
-        </is>
-      </c>
-      <c r="B4" s="35" t="inlineStr">
-        <is>
-          <t>Dr. Levi — Maccabi</t>
-        </is>
-      </c>
-      <c r="C4" s="35" t="inlineStr">
-        <is>
-          <t>Family doctor</t>
-        </is>
-      </c>
-      <c r="D4" s="36" t="n">
-        <v>45966</v>
-      </c>
-      <c r="E4" s="36" t="n">
-        <v>46331</v>
-      </c>
-      <c r="F4" s="35" t="inlineStr">
-        <is>
-          <t>Yearly</t>
-        </is>
-      </c>
-      <c r="G4" s="35" t="n"/>
-      <c r="H4" s="35" t="inlineStr">
-        <is>
-          <t>[clinic phone]</t>
-        </is>
-      </c>
-      <c r="I4" s="35" t="n"/>
-    </row>
-    <row r="5" ht="36" customHeight="1" s="28">
-      <c r="A5" s="35" t="inlineStr">
-        <is>
-          <t>[Child 1]</t>
-        </is>
-      </c>
-      <c r="B5" s="35" t="inlineStr">
-        <is>
-          <t>Dr. Cohen — Clalit</t>
-        </is>
-      </c>
-      <c r="C5" s="35" t="inlineStr">
-        <is>
-          <t>Pediatrician</t>
-        </is>
-      </c>
-      <c r="D5" s="36" t="n">
-        <v>46101</v>
-      </c>
-      <c r="E5" s="36" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F5" s="35" t="inlineStr">
-        <is>
-          <t>6-month</t>
-        </is>
-      </c>
-      <c r="G5" s="35" t="inlineStr">
-        <is>
-          <t>Routine check</t>
-        </is>
-      </c>
-      <c r="H5" s="35" t="inlineStr">
-        <is>
-          <t>[clinic phone]</t>
-        </is>
-      </c>
-      <c r="I5" s="35" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1" s="28">
-      <c r="A6" s="35" t="inlineStr">
-        <is>
-          <t>[Child 1]</t>
-        </is>
-      </c>
-      <c r="B6" s="35" t="inlineStr">
-        <is>
-          <t>Tipat Halav</t>
-        </is>
-      </c>
-      <c r="C6" s="35" t="inlineStr">
-        <is>
-          <t>Vaccines</t>
-        </is>
-      </c>
-      <c r="D6" s="36" t="n">
-        <v>46113</v>
-      </c>
-      <c r="E6" s="36" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F6" s="35" t="inlineStr">
-        <is>
-          <t>Per schedule</t>
-        </is>
-      </c>
-      <c r="G6" s="35" t="inlineStr">
-        <is>
-          <t>MMR booster</t>
-        </is>
-      </c>
-      <c r="H6" s="35" t="inlineStr">
-        <is>
-          <t>[Tipat Halav phone]</t>
-        </is>
-      </c>
-      <c r="I6" s="35" t="n"/>
-    </row>
-    <row r="7" ht="36" customHeight="1" s="28">
-      <c r="A7" s="35" t="inlineStr">
-        <is>
-          <t>[Child 2]</t>
-        </is>
-      </c>
-      <c r="B7" s="35" t="inlineStr">
-        <is>
-          <t>Tipat Halav</t>
-        </is>
-      </c>
-      <c r="C7" s="35" t="inlineStr">
-        <is>
-          <t>Vaccines</t>
-        </is>
-      </c>
-      <c r="D7" s="36" t="n">
-        <v>46063</v>
-      </c>
-      <c r="E7" s="36" t="n">
-        <v>46244</v>
-      </c>
-      <c r="F7" s="35" t="inlineStr">
-        <is>
-          <t>Per schedule</t>
-        </is>
-      </c>
-      <c r="G7" s="35" t="inlineStr">
-        <is>
-          <t>12-month vaccines</t>
-        </is>
-      </c>
-      <c r="H7" s="35" t="inlineStr">
-        <is>
-          <t>[Tipat Halav phone]</t>
-        </is>
-      </c>
-      <c r="I7" s="35" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="28">
-      <c r="A8" s="37" t="n"/>
-      <c r="B8" s="37" t="n"/>
-      <c r="C8" s="37" t="n"/>
-      <c r="D8" s="37" t="n"/>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="37" t="n"/>
-      <c r="G8" s="37" t="n"/>
-      <c r="H8" s="37" t="n"/>
-      <c r="I8" s="37" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="28">
-      <c r="A9" s="37" t="n"/>
-      <c r="B9" s="37" t="n"/>
-      <c r="C9" s="37" t="n"/>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="37" t="n"/>
-      <c r="G9" s="37" t="n"/>
-      <c r="H9" s="37" t="n"/>
-      <c r="I9" s="37" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="28">
-      <c r="A10" s="37" t="n"/>
-      <c r="B10" s="37" t="n"/>
-      <c r="C10" s="37" t="n"/>
-      <c r="D10" s="37" t="n"/>
-      <c r="E10" s="37" t="n"/>
-      <c r="F10" s="37" t="n"/>
-      <c r="G10" s="37" t="n"/>
-      <c r="H10" s="37" t="n"/>
-      <c r="I10" s="37" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="28">
-      <c r="A11" s="37" t="n"/>
-      <c r="B11" s="37" t="n"/>
-      <c r="C11" s="37" t="n"/>
-      <c r="D11" s="37" t="n"/>
-      <c r="E11" s="37" t="n"/>
-      <c r="F11" s="37" t="n"/>
-      <c r="G11" s="37" t="n"/>
-      <c r="H11" s="37" t="n"/>
-      <c r="I11" s="37" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="28">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="37" t="n"/>
-      <c r="C12" s="37" t="n"/>
-      <c r="D12" s="37" t="n"/>
-      <c r="E12" s="37" t="n"/>
-      <c r="F12" s="37" t="n"/>
-      <c r="G12" s="37" t="n"/>
-      <c r="H12" s="37" t="n"/>
-      <c r="I12" s="37" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="28">
-      <c r="A13" s="37" t="n"/>
-      <c r="B13" s="37" t="n"/>
-      <c r="C13" s="37" t="n"/>
-      <c r="D13" s="37" t="n"/>
-      <c r="E13" s="37" t="n"/>
-      <c r="F13" s="37" t="n"/>
-      <c r="G13" s="37" t="n"/>
-      <c r="H13" s="37" t="n"/>
-      <c r="I13" s="37" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="28">
-      <c r="A14" s="37" t="n"/>
-      <c r="B14" s="37" t="n"/>
-      <c r="C14" s="37" t="n"/>
-      <c r="D14" s="37" t="n"/>
-      <c r="E14" s="37" t="n"/>
-      <c r="F14" s="37" t="n"/>
-      <c r="G14" s="37" t="n"/>
-      <c r="H14" s="37" t="n"/>
-      <c r="I14" s="37" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="28">
-      <c r="A15" s="37" t="n"/>
-      <c r="B15" s="37" t="n"/>
-      <c r="C15" s="37" t="n"/>
-      <c r="D15" s="37" t="n"/>
-      <c r="E15" s="37" t="n"/>
-      <c r="F15" s="37" t="n"/>
-      <c r="G15" s="37" t="n"/>
-      <c r="H15" s="37" t="n"/>
-      <c r="I15" s="37" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="28">
-      <c r="A16" s="37" t="n"/>
-      <c r="B16" s="37" t="n"/>
-      <c r="C16" s="37" t="n"/>
-      <c r="D16" s="37" t="n"/>
-      <c r="E16" s="37" t="n"/>
-      <c r="F16" s="37" t="n"/>
-      <c r="G16" s="37" t="n"/>
-      <c r="H16" s="37" t="n"/>
-      <c r="I16" s="37" t="n"/>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="28">
-      <c r="A17" s="37" t="n"/>
-      <c r="B17" s="37" t="n"/>
-      <c r="C17" s="37" t="n"/>
-      <c r="D17" s="37" t="n"/>
-      <c r="E17" s="37" t="n"/>
-      <c r="F17" s="37" t="n"/>
-      <c r="G17" s="37" t="n"/>
-      <c r="H17" s="37" t="n"/>
-      <c r="I17" s="37" t="n"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="28">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="37" t="n"/>
-      <c r="C18" s="37" t="n"/>
-      <c r="D18" s="37" t="n"/>
-      <c r="E18" s="37" t="n"/>
-      <c r="F18" s="37" t="n"/>
-      <c r="G18" s="37" t="n"/>
-      <c r="H18" s="37" t="n"/>
-      <c r="I18" s="37" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="28">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="37" t="n"/>
-      <c r="C19" s="37" t="n"/>
-      <c r="D19" s="37" t="n"/>
-      <c r="E19" s="37" t="n"/>
-      <c r="F19" s="37" t="n"/>
-      <c r="G19" s="37" t="n"/>
-      <c r="H19" s="37" t="n"/>
-      <c r="I19" s="37" t="n"/>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="28">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="37" t="n"/>
-      <c r="C20" s="37" t="n"/>
-      <c r="D20" s="37" t="n"/>
-      <c r="E20" s="37" t="n"/>
-      <c r="F20" s="37" t="n"/>
-      <c r="G20" s="37" t="n"/>
-      <c r="H20" s="37" t="n"/>
-      <c r="I20" s="37" t="n"/>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="28">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="37" t="n"/>
-      <c r="C21" s="37" t="n"/>
-      <c r="D21" s="37" t="n"/>
-      <c r="E21" s="37" t="n"/>
-      <c r="F21" s="37" t="n"/>
-      <c r="G21" s="37" t="n"/>
-      <c r="H21" s="37" t="n"/>
-      <c r="I21" s="37" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="28">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="37" t="n"/>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="37" t="n"/>
-      <c r="G22" s="37" t="n"/>
-      <c r="H22" s="37" t="n"/>
-      <c r="I22" s="37" t="n"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="E2:E1000">
-    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="4" text="" percent="0" bottom="0">
-      <formula>AND(ISNUMBER(E2),E2&lt;TODAY())</formula>
-    </cfRule>
-    <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="0" text="" percent="0" bottom="0">
-      <formula>AND(ISNUMBER(E2),E2-TODAY()&gt;=0,E2-TODAY()&lt;=30)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2009,7 +1636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2378,7 +2005,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2865,7 +2492,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3490,7 +3117,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3500,50 +3127,146 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>you@example.com</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>Adar</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>partner@example.com</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>Shanee</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>lang</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>he</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>msg_id</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>group_name</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>group_type</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>sender_name</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>sender_role</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>received_at</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>has_media</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>one_liner</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>action_required</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>action_owner</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>dispatched</t>
+        </is>
+      </c>
+      <c r="O1" s="27" t="inlineStr">
+        <is>
+          <t>dispatched_at</t>
+        </is>
+      </c>
+      <c r="P1" s="27" t="inlineStr">
+        <is>
+          <t>digested_at</t>
         </is>
       </c>
     </row>
@@ -3558,88 +3281,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>msg_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>group_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>group_type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>sender_name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>sender_role</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>received_at</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>has_media</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>classification</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
+      <c r="F1" s="27" t="inlineStr">
         <is>
           <t>one_liner</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>action_required</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>action_owner</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dispatched</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>dispatched_at</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>digested_at</t>
         </is>
       </c>
     </row>
@@ -3654,38 +3327,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>msg_id</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>group_name</t>
+          <t>Account</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sender_name</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>received_at</t>
+          <t>Amount (ILS)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>one_liner</t>
+          <t>Cat-Source</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Txn-ID</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Imported-At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>[Joint Checking]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SHUFERSAL DEAL</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-432.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>sample-1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-11T06:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[Visa Cal — Adar]</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PAZ GAS STATION</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-280</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>sample-2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-11T06:00:00</t>
         </is>
       </c>
     </row>
@@ -4717,22 +4480,22 @@
           <t>Auto-flag</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="27" t="inlineStr">
         <is>
           <t>LastDoneBy</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="27" t="inlineStr">
         <is>
           <t>DoneAt</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="27" t="inlineStr">
         <is>
           <t>WriteQueue_Tombstone</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="27" t="inlineStr">
         <is>
           <t>Guide URL</t>
         </is>
@@ -5926,1124 +5689,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="12" customWidth="1" style="27" min="1" max="1"/>
-    <col width="22" customWidth="1" style="27" min="2" max="2"/>
-    <col width="36" customWidth="1" style="27" min="3" max="3"/>
-    <col width="14" customWidth="1" style="27" min="4" max="4"/>
-    <col width="16" customWidth="1" style="27" min="5" max="7"/>
-    <col width="22" customWidth="1" style="27" min="8" max="8"/>
-    <col width="24" customWidth="1" style="27" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="27.75" customHeight="1" s="28">
-      <c r="A1" s="34" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="34" t="inlineStr">
-        <is>
-          <t>Account</t>
-        </is>
-      </c>
-      <c r="C1" s="34" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D1" s="34" t="inlineStr">
-        <is>
-          <t>Amount (ILS)</t>
-        </is>
-      </c>
-      <c r="E1" s="34" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="F1" s="34" t="inlineStr">
-        <is>
-          <t>Subcategory</t>
-        </is>
-      </c>
-      <c r="G1" s="34" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="H1" s="34" t="inlineStr">
-        <is>
-          <t>Imported From</t>
-        </is>
-      </c>
-      <c r="I1" s="34" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1" s="28">
-      <c r="A2" s="36" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B2" s="35" t="inlineStr">
-        <is>
-          <t>[Joint Checking]</t>
-        </is>
-      </c>
-      <c r="C2" s="35" t="inlineStr">
-        <is>
-          <t>SHUFERSAL DEAL</t>
-        </is>
-      </c>
-      <c r="D2" s="42" t="n">
-        <v>-432.5</v>
-      </c>
-      <c r="E2" s="35" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
-      </c>
-      <c r="F2" s="35" t="inlineStr">
-        <is>
-          <t>Supermarket</t>
-        </is>
-      </c>
-      <c r="G2" s="35" t="inlineStr">
-        <is>
-          <t>kids</t>
-        </is>
-      </c>
-      <c r="H2" s="35" t="inlineStr">
-        <is>
-          <t>hapoalim_2026-05.csv</t>
-        </is>
-      </c>
-      <c r="I2" s="35" t="inlineStr">
-        <is>
-          <t>Sample row</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1" s="28">
-      <c r="A3" s="36" t="n">
-        <v>46154</v>
-      </c>
-      <c r="B3" s="35" t="inlineStr">
-        <is>
-          <t>[Visa Cal — Adar]</t>
-        </is>
-      </c>
-      <c r="C3" s="35" t="inlineStr">
-        <is>
-          <t>PAZ GAS STATION</t>
-        </is>
-      </c>
-      <c r="D3" s="42" t="n">
-        <v>-280</v>
-      </c>
-      <c r="E3" s="35" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="F3" s="35" t="inlineStr">
-        <is>
-          <t>Fuel</t>
-        </is>
-      </c>
-      <c r="G3" s="35" t="inlineStr">
-        <is>
-          <t>car</t>
-        </is>
-      </c>
-      <c r="H3" s="35" t="inlineStr">
-        <is>
-          <t>cal_2026-05.csv</t>
-        </is>
-      </c>
-      <c r="I3" s="35" t="n"/>
-    </row>
-    <row r="4" ht="36" customHeight="1" s="28">
-      <c r="A4" s="36" t="n">
-        <v>46157</v>
-      </c>
-      <c r="B4" s="35" t="inlineStr">
-        <is>
-          <t>[Joint Checking]</t>
-        </is>
-      </c>
-      <c r="C4" s="35" t="inlineStr">
-        <is>
-          <t>MORTGAGE PAYMENT</t>
-        </is>
-      </c>
-      <c r="D4" s="42" t="n">
-        <v>-6800</v>
-      </c>
-      <c r="E4" s="35" t="inlineStr">
-        <is>
-          <t>Housing</t>
-        </is>
-      </c>
-      <c r="F4" s="35" t="inlineStr">
-        <is>
-          <t>Mortgage</t>
-        </is>
-      </c>
-      <c r="G4" s="35" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="H4" s="35" t="inlineStr">
-        <is>
-          <t>hapoalim_2026-05.csv</t>
-        </is>
-      </c>
-      <c r="I4" s="35" t="n"/>
-    </row>
-    <row r="5" ht="36" customHeight="1" s="28">
-      <c r="A5" s="36" t="n">
-        <v>46162</v>
-      </c>
-      <c r="B5" s="35" t="inlineStr">
-        <is>
-          <t>[Joint Checking]</t>
-        </is>
-      </c>
-      <c r="C5" s="35" t="inlineStr">
-        <is>
-          <t>SALARY — ADAR</t>
-        </is>
-      </c>
-      <c r="D5" s="42" t="n">
-        <v>28500</v>
-      </c>
-      <c r="E5" s="35" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="F5" s="35" t="inlineStr">
-        <is>
-          <t>Salary</t>
-        </is>
-      </c>
-      <c r="G5" s="35" t="inlineStr">
-        <is>
-          <t>income</t>
-        </is>
-      </c>
-      <c r="H5" s="35" t="inlineStr">
-        <is>
-          <t>hapoalim_2026-05.csv</t>
-        </is>
-      </c>
-      <c r="I5" s="35" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="28">
-      <c r="A6" s="37" t="n"/>
-      <c r="B6" s="37" t="n"/>
-      <c r="C6" s="37" t="n"/>
-      <c r="D6" s="43" t="n"/>
-      <c r="E6" s="37" t="n"/>
-      <c r="F6" s="37" t="n"/>
-      <c r="G6" s="37" t="n"/>
-      <c r="H6" s="37" t="n"/>
-      <c r="I6" s="37" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="28">
-      <c r="A7" s="37" t="n"/>
-      <c r="B7" s="37" t="n"/>
-      <c r="C7" s="37" t="n"/>
-      <c r="D7" s="43" t="n"/>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="37" t="n"/>
-      <c r="G7" s="37" t="n"/>
-      <c r="H7" s="37" t="n"/>
-      <c r="I7" s="37" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="28">
-      <c r="A8" s="37" t="n"/>
-      <c r="B8" s="37" t="n"/>
-      <c r="C8" s="37" t="n"/>
-      <c r="D8" s="43" t="n"/>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="37" t="n"/>
-      <c r="G8" s="37" t="n"/>
-      <c r="H8" s="37" t="n"/>
-      <c r="I8" s="37" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="28">
-      <c r="A9" s="37" t="n"/>
-      <c r="B9" s="37" t="n"/>
-      <c r="C9" s="37" t="n"/>
-      <c r="D9" s="43" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="37" t="n"/>
-      <c r="G9" s="37" t="n"/>
-      <c r="H9" s="37" t="n"/>
-      <c r="I9" s="37" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="28">
-      <c r="A10" s="37" t="n"/>
-      <c r="B10" s="37" t="n"/>
-      <c r="C10" s="37" t="n"/>
-      <c r="D10" s="43" t="n"/>
-      <c r="E10" s="37" t="n"/>
-      <c r="F10" s="37" t="n"/>
-      <c r="G10" s="37" t="n"/>
-      <c r="H10" s="37" t="n"/>
-      <c r="I10" s="37" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="28">
-      <c r="A11" s="37" t="n"/>
-      <c r="B11" s="37" t="n"/>
-      <c r="C11" s="37" t="n"/>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="37" t="n"/>
-      <c r="F11" s="37" t="n"/>
-      <c r="G11" s="37" t="n"/>
-      <c r="H11" s="37" t="n"/>
-      <c r="I11" s="37" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="28">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="37" t="n"/>
-      <c r="C12" s="37" t="n"/>
-      <c r="D12" s="43" t="n"/>
-      <c r="E12" s="37" t="n"/>
-      <c r="F12" s="37" t="n"/>
-      <c r="G12" s="37" t="n"/>
-      <c r="H12" s="37" t="n"/>
-      <c r="I12" s="37" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="28">
-      <c r="A13" s="37" t="n"/>
-      <c r="B13" s="37" t="n"/>
-      <c r="C13" s="37" t="n"/>
-      <c r="D13" s="43" t="n"/>
-      <c r="E13" s="37" t="n"/>
-      <c r="F13" s="37" t="n"/>
-      <c r="G13" s="37" t="n"/>
-      <c r="H13" s="37" t="n"/>
-      <c r="I13" s="37" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="28">
-      <c r="A14" s="37" t="n"/>
-      <c r="B14" s="37" t="n"/>
-      <c r="C14" s="37" t="n"/>
-      <c r="D14" s="43" t="n"/>
-      <c r="E14" s="37" t="n"/>
-      <c r="F14" s="37" t="n"/>
-      <c r="G14" s="37" t="n"/>
-      <c r="H14" s="37" t="n"/>
-      <c r="I14" s="37" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="28">
-      <c r="A15" s="37" t="n"/>
-      <c r="B15" s="37" t="n"/>
-      <c r="C15" s="37" t="n"/>
-      <c r="D15" s="43" t="n"/>
-      <c r="E15" s="37" t="n"/>
-      <c r="F15" s="37" t="n"/>
-      <c r="G15" s="37" t="n"/>
-      <c r="H15" s="37" t="n"/>
-      <c r="I15" s="37" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="28">
-      <c r="A16" s="37" t="n"/>
-      <c r="B16" s="37" t="n"/>
-      <c r="C16" s="37" t="n"/>
-      <c r="D16" s="43" t="n"/>
-      <c r="E16" s="37" t="n"/>
-      <c r="F16" s="37" t="n"/>
-      <c r="G16" s="37" t="n"/>
-      <c r="H16" s="37" t="n"/>
-      <c r="I16" s="37" t="n"/>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="28">
-      <c r="A17" s="37" t="n"/>
-      <c r="B17" s="37" t="n"/>
-      <c r="C17" s="37" t="n"/>
-      <c r="D17" s="43" t="n"/>
-      <c r="E17" s="37" t="n"/>
-      <c r="F17" s="37" t="n"/>
-      <c r="G17" s="37" t="n"/>
-      <c r="H17" s="37" t="n"/>
-      <c r="I17" s="37" t="n"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="28">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="37" t="n"/>
-      <c r="C18" s="37" t="n"/>
-      <c r="D18" s="43" t="n"/>
-      <c r="E18" s="37" t="n"/>
-      <c r="F18" s="37" t="n"/>
-      <c r="G18" s="37" t="n"/>
-      <c r="H18" s="37" t="n"/>
-      <c r="I18" s="37" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="28">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="37" t="n"/>
-      <c r="C19" s="37" t="n"/>
-      <c r="D19" s="43" t="n"/>
-      <c r="E19" s="37" t="n"/>
-      <c r="F19" s="37" t="n"/>
-      <c r="G19" s="37" t="n"/>
-      <c r="H19" s="37" t="n"/>
-      <c r="I19" s="37" t="n"/>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="28">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="37" t="n"/>
-      <c r="C20" s="37" t="n"/>
-      <c r="D20" s="43" t="n"/>
-      <c r="E20" s="37" t="n"/>
-      <c r="F20" s="37" t="n"/>
-      <c r="G20" s="37" t="n"/>
-      <c r="H20" s="37" t="n"/>
-      <c r="I20" s="37" t="n"/>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="28">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="37" t="n"/>
-      <c r="C21" s="37" t="n"/>
-      <c r="D21" s="43" t="n"/>
-      <c r="E21" s="37" t="n"/>
-      <c r="F21" s="37" t="n"/>
-      <c r="G21" s="37" t="n"/>
-      <c r="H21" s="37" t="n"/>
-      <c r="I21" s="37" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="28">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="37" t="n"/>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="43" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="37" t="n"/>
-      <c r="G22" s="37" t="n"/>
-      <c r="H22" s="37" t="n"/>
-      <c r="I22" s="37" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="28">
-      <c r="A23" s="37" t="n"/>
-      <c r="B23" s="37" t="n"/>
-      <c r="C23" s="37" t="n"/>
-      <c r="D23" s="43" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="37" t="n"/>
-      <c r="G23" s="37" t="n"/>
-      <c r="H23" s="37" t="n"/>
-      <c r="I23" s="37" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="28">
-      <c r="A24" s="37" t="n"/>
-      <c r="B24" s="37" t="n"/>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="43" t="n"/>
-      <c r="E24" s="37" t="n"/>
-      <c r="F24" s="37" t="n"/>
-      <c r="G24" s="37" t="n"/>
-      <c r="H24" s="37" t="n"/>
-      <c r="I24" s="37" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="28">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="n"/>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="43" t="n"/>
-      <c r="E25" s="37" t="n"/>
-      <c r="F25" s="37" t="n"/>
-      <c r="G25" s="37" t="n"/>
-      <c r="H25" s="37" t="n"/>
-      <c r="I25" s="37" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="28">
-      <c r="A26" s="37" t="n"/>
-      <c r="B26" s="37" t="n"/>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="43" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="37" t="n"/>
-      <c r="G26" s="37" t="n"/>
-      <c r="H26" s="37" t="n"/>
-      <c r="I26" s="37" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="28">
-      <c r="A27" s="37" t="n"/>
-      <c r="B27" s="37" t="n"/>
-      <c r="C27" s="37" t="n"/>
-      <c r="D27" s="43" t="n"/>
-      <c r="E27" s="37" t="n"/>
-      <c r="F27" s="37" t="n"/>
-      <c r="G27" s="37" t="n"/>
-      <c r="H27" s="37" t="n"/>
-      <c r="I27" s="37" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="28">
-      <c r="A28" s="37" t="n"/>
-      <c r="B28" s="37" t="n"/>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="43" t="n"/>
-      <c r="E28" s="37" t="n"/>
-      <c r="F28" s="37" t="n"/>
-      <c r="G28" s="37" t="n"/>
-      <c r="H28" s="37" t="n"/>
-      <c r="I28" s="37" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="28">
-      <c r="A29" s="37" t="n"/>
-      <c r="B29" s="37" t="n"/>
-      <c r="C29" s="37" t="n"/>
-      <c r="D29" s="43" t="n"/>
-      <c r="E29" s="37" t="n"/>
-      <c r="F29" s="37" t="n"/>
-      <c r="G29" s="37" t="n"/>
-      <c r="H29" s="37" t="n"/>
-      <c r="I29" s="37" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="28">
-      <c r="A30" s="37" t="n"/>
-      <c r="B30" s="37" t="n"/>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="43" t="n"/>
-      <c r="E30" s="37" t="n"/>
-      <c r="F30" s="37" t="n"/>
-      <c r="G30" s="37" t="n"/>
-      <c r="H30" s="37" t="n"/>
-      <c r="I30" s="37" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="28">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="37" t="n"/>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="43" t="n"/>
-      <c r="E31" s="37" t="n"/>
-      <c r="F31" s="37" t="n"/>
-      <c r="G31" s="37" t="n"/>
-      <c r="H31" s="37" t="n"/>
-      <c r="I31" s="37" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="28">
-      <c r="A32" s="37" t="n"/>
-      <c r="B32" s="37" t="n"/>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="43" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="37" t="n"/>
-      <c r="G32" s="37" t="n"/>
-      <c r="H32" s="37" t="n"/>
-      <c r="I32" s="37" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="28">
-      <c r="A33" s="37" t="n"/>
-      <c r="B33" s="37" t="n"/>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="43" t="n"/>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="37" t="n"/>
-      <c r="G33" s="37" t="n"/>
-      <c r="H33" s="37" t="n"/>
-      <c r="I33" s="37" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="28">
-      <c r="A34" s="37" t="n"/>
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="43" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="37" t="n"/>
-      <c r="G34" s="37" t="n"/>
-      <c r="H34" s="37" t="n"/>
-      <c r="I34" s="37" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="28">
-      <c r="A35" s="37" t="n"/>
-      <c r="B35" s="37" t="n"/>
-      <c r="C35" s="37" t="n"/>
-      <c r="D35" s="43" t="n"/>
-      <c r="E35" s="37" t="n"/>
-      <c r="F35" s="37" t="n"/>
-      <c r="G35" s="37" t="n"/>
-      <c r="H35" s="37" t="n"/>
-      <c r="I35" s="37" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="28">
-      <c r="A36" s="37" t="n"/>
-      <c r="B36" s="37" t="n"/>
-      <c r="C36" s="37" t="n"/>
-      <c r="D36" s="43" t="n"/>
-      <c r="E36" s="37" t="n"/>
-      <c r="F36" s="37" t="n"/>
-      <c r="G36" s="37" t="n"/>
-      <c r="H36" s="37" t="n"/>
-      <c r="I36" s="37" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="28">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="43" t="n"/>
-      <c r="E37" s="37" t="n"/>
-      <c r="F37" s="37" t="n"/>
-      <c r="G37" s="37" t="n"/>
-      <c r="H37" s="37" t="n"/>
-      <c r="I37" s="37" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="28">
-      <c r="A38" s="37" t="n"/>
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="37" t="n"/>
-      <c r="D38" s="43" t="n"/>
-      <c r="E38" s="37" t="n"/>
-      <c r="F38" s="37" t="n"/>
-      <c r="G38" s="37" t="n"/>
-      <c r="H38" s="37" t="n"/>
-      <c r="I38" s="37" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="28">
-      <c r="A39" s="37" t="n"/>
-      <c r="B39" s="37" t="n"/>
-      <c r="C39" s="37" t="n"/>
-      <c r="D39" s="43" t="n"/>
-      <c r="E39" s="37" t="n"/>
-      <c r="F39" s="37" t="n"/>
-      <c r="G39" s="37" t="n"/>
-      <c r="H39" s="37" t="n"/>
-      <c r="I39" s="37" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="28">
-      <c r="A40" s="37" t="n"/>
-      <c r="B40" s="37" t="n"/>
-      <c r="C40" s="37" t="n"/>
-      <c r="D40" s="43" t="n"/>
-      <c r="E40" s="37" t="n"/>
-      <c r="F40" s="37" t="n"/>
-      <c r="G40" s="37" t="n"/>
-      <c r="H40" s="37" t="n"/>
-      <c r="I40" s="37" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="28">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="37" t="n"/>
-      <c r="C41" s="37" t="n"/>
-      <c r="D41" s="43" t="n"/>
-      <c r="E41" s="37" t="n"/>
-      <c r="F41" s="37" t="n"/>
-      <c r="G41" s="37" t="n"/>
-      <c r="H41" s="37" t="n"/>
-      <c r="I41" s="37" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="28">
-      <c r="A42" s="37" t="n"/>
-      <c r="B42" s="37" t="n"/>
-      <c r="C42" s="37" t="n"/>
-      <c r="D42" s="43" t="n"/>
-      <c r="E42" s="37" t="n"/>
-      <c r="F42" s="37" t="n"/>
-      <c r="G42" s="37" t="n"/>
-      <c r="H42" s="37" t="n"/>
-      <c r="I42" s="37" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="28">
-      <c r="A43" s="37" t="n"/>
-      <c r="B43" s="37" t="n"/>
-      <c r="C43" s="37" t="n"/>
-      <c r="D43" s="43" t="n"/>
-      <c r="E43" s="37" t="n"/>
-      <c r="F43" s="37" t="n"/>
-      <c r="G43" s="37" t="n"/>
-      <c r="H43" s="37" t="n"/>
-      <c r="I43" s="37" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="28">
-      <c r="A44" s="37" t="n"/>
-      <c r="B44" s="37" t="n"/>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="43" t="n"/>
-      <c r="E44" s="37" t="n"/>
-      <c r="F44" s="37" t="n"/>
-      <c r="G44" s="37" t="n"/>
-      <c r="H44" s="37" t="n"/>
-      <c r="I44" s="37" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="28">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="n"/>
-      <c r="C45" s="37" t="n"/>
-      <c r="D45" s="43" t="n"/>
-      <c r="E45" s="37" t="n"/>
-      <c r="F45" s="37" t="n"/>
-      <c r="G45" s="37" t="n"/>
-      <c r="H45" s="37" t="n"/>
-      <c r="I45" s="37" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="28">
-      <c r="A46" s="37" t="n"/>
-      <c r="B46" s="37" t="n"/>
-      <c r="C46" s="37" t="n"/>
-      <c r="D46" s="43" t="n"/>
-      <c r="E46" s="37" t="n"/>
-      <c r="F46" s="37" t="n"/>
-      <c r="G46" s="37" t="n"/>
-      <c r="H46" s="37" t="n"/>
-      <c r="I46" s="37" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="28">
-      <c r="A47" s="37" t="n"/>
-      <c r="B47" s="37" t="n"/>
-      <c r="C47" s="37" t="n"/>
-      <c r="D47" s="43" t="n"/>
-      <c r="E47" s="37" t="n"/>
-      <c r="F47" s="37" t="n"/>
-      <c r="G47" s="37" t="n"/>
-      <c r="H47" s="37" t="n"/>
-      <c r="I47" s="37" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="28">
-      <c r="A48" s="37" t="n"/>
-      <c r="B48" s="37" t="n"/>
-      <c r="C48" s="37" t="n"/>
-      <c r="D48" s="43" t="n"/>
-      <c r="E48" s="37" t="n"/>
-      <c r="F48" s="37" t="n"/>
-      <c r="G48" s="37" t="n"/>
-      <c r="H48" s="37" t="n"/>
-      <c r="I48" s="37" t="n"/>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="28">
-      <c r="A49" s="37" t="n"/>
-      <c r="B49" s="37" t="n"/>
-      <c r="C49" s="37" t="n"/>
-      <c r="D49" s="43" t="n"/>
-      <c r="E49" s="37" t="n"/>
-      <c r="F49" s="37" t="n"/>
-      <c r="G49" s="37" t="n"/>
-      <c r="H49" s="37" t="n"/>
-      <c r="I49" s="37" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="28">
-      <c r="A50" s="37" t="n"/>
-      <c r="B50" s="37" t="n"/>
-      <c r="C50" s="37" t="n"/>
-      <c r="D50" s="43" t="n"/>
-      <c r="E50" s="37" t="n"/>
-      <c r="F50" s="37" t="n"/>
-      <c r="G50" s="37" t="n"/>
-      <c r="H50" s="37" t="n"/>
-      <c r="I50" s="37" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="28">
-      <c r="A51" s="37" t="n"/>
-      <c r="B51" s="37" t="n"/>
-      <c r="C51" s="37" t="n"/>
-      <c r="D51" s="43" t="n"/>
-      <c r="E51" s="37" t="n"/>
-      <c r="F51" s="37" t="n"/>
-      <c r="G51" s="37" t="n"/>
-      <c r="H51" s="37" t="n"/>
-      <c r="I51" s="37" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="28">
-      <c r="A52" s="37" t="n"/>
-      <c r="B52" s="37" t="n"/>
-      <c r="C52" s="37" t="n"/>
-      <c r="D52" s="43" t="n"/>
-      <c r="E52" s="37" t="n"/>
-      <c r="F52" s="37" t="n"/>
-      <c r="G52" s="37" t="n"/>
-      <c r="H52" s="37" t="n"/>
-      <c r="I52" s="37" t="n"/>
-    </row>
-    <row r="53" ht="15" customHeight="1" s="28">
-      <c r="A53" s="37" t="n"/>
-      <c r="B53" s="37" t="n"/>
-      <c r="C53" s="37" t="n"/>
-      <c r="D53" s="43" t="n"/>
-      <c r="E53" s="37" t="n"/>
-      <c r="F53" s="37" t="n"/>
-      <c r="G53" s="37" t="n"/>
-      <c r="H53" s="37" t="n"/>
-      <c r="I53" s="37" t="n"/>
-    </row>
-    <row r="54" ht="15" customHeight="1" s="28">
-      <c r="A54" s="37" t="n"/>
-      <c r="B54" s="37" t="n"/>
-      <c r="C54" s="37" t="n"/>
-      <c r="D54" s="43" t="n"/>
-      <c r="E54" s="37" t="n"/>
-      <c r="F54" s="37" t="n"/>
-      <c r="G54" s="37" t="n"/>
-      <c r="H54" s="37" t="n"/>
-      <c r="I54" s="37" t="n"/>
-    </row>
-    <row r="55" ht="15" customHeight="1" s="28">
-      <c r="A55" s="37" t="n"/>
-      <c r="B55" s="37" t="n"/>
-      <c r="C55" s="37" t="n"/>
-      <c r="D55" s="43" t="n"/>
-      <c r="E55" s="37" t="n"/>
-      <c r="F55" s="37" t="n"/>
-      <c r="G55" s="37" t="n"/>
-      <c r="H55" s="37" t="n"/>
-      <c r="I55" s="37" t="n"/>
-    </row>
-    <row r="56" ht="15" customHeight="1" s="28">
-      <c r="A56" s="37" t="n"/>
-      <c r="B56" s="37" t="n"/>
-      <c r="C56" s="37" t="n"/>
-      <c r="D56" s="43" t="n"/>
-      <c r="E56" s="37" t="n"/>
-      <c r="F56" s="37" t="n"/>
-      <c r="G56" s="37" t="n"/>
-      <c r="H56" s="37" t="n"/>
-      <c r="I56" s="37" t="n"/>
-    </row>
-    <row r="57" ht="15" customHeight="1" s="28">
-      <c r="A57" s="37" t="n"/>
-      <c r="B57" s="37" t="n"/>
-      <c r="C57" s="37" t="n"/>
-      <c r="D57" s="43" t="n"/>
-      <c r="E57" s="37" t="n"/>
-      <c r="F57" s="37" t="n"/>
-      <c r="G57" s="37" t="n"/>
-      <c r="H57" s="37" t="n"/>
-      <c r="I57" s="37" t="n"/>
-    </row>
-    <row r="58" ht="15" customHeight="1" s="28">
-      <c r="A58" s="37" t="n"/>
-      <c r="B58" s="37" t="n"/>
-      <c r="C58" s="37" t="n"/>
-      <c r="D58" s="43" t="n"/>
-      <c r="E58" s="37" t="n"/>
-      <c r="F58" s="37" t="n"/>
-      <c r="G58" s="37" t="n"/>
-      <c r="H58" s="37" t="n"/>
-      <c r="I58" s="37" t="n"/>
-    </row>
-    <row r="59" ht="15" customHeight="1" s="28">
-      <c r="A59" s="37" t="n"/>
-      <c r="B59" s="37" t="n"/>
-      <c r="C59" s="37" t="n"/>
-      <c r="D59" s="43" t="n"/>
-      <c r="E59" s="37" t="n"/>
-      <c r="F59" s="37" t="n"/>
-      <c r="G59" s="37" t="n"/>
-      <c r="H59" s="37" t="n"/>
-      <c r="I59" s="37" t="n"/>
-    </row>
-    <row r="60" ht="15" customHeight="1" s="28">
-      <c r="A60" s="37" t="n"/>
-      <c r="B60" s="37" t="n"/>
-      <c r="C60" s="37" t="n"/>
-      <c r="D60" s="43" t="n"/>
-      <c r="E60" s="37" t="n"/>
-      <c r="F60" s="37" t="n"/>
-      <c r="G60" s="37" t="n"/>
-      <c r="H60" s="37" t="n"/>
-      <c r="I60" s="37" t="n"/>
-    </row>
-    <row r="61" ht="15" customHeight="1" s="28">
-      <c r="A61" s="37" t="n"/>
-      <c r="B61" s="37" t="n"/>
-      <c r="C61" s="37" t="n"/>
-      <c r="D61" s="43" t="n"/>
-      <c r="E61" s="37" t="n"/>
-      <c r="F61" s="37" t="n"/>
-      <c r="G61" s="37" t="n"/>
-      <c r="H61" s="37" t="n"/>
-      <c r="I61" s="37" t="n"/>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="28">
-      <c r="A62" s="37" t="n"/>
-      <c r="B62" s="37" t="n"/>
-      <c r="C62" s="37" t="n"/>
-      <c r="D62" s="43" t="n"/>
-      <c r="E62" s="37" t="n"/>
-      <c r="F62" s="37" t="n"/>
-      <c r="G62" s="37" t="n"/>
-      <c r="H62" s="37" t="n"/>
-      <c r="I62" s="37" t="n"/>
-    </row>
-    <row r="63" ht="15" customHeight="1" s="28">
-      <c r="A63" s="37" t="n"/>
-      <c r="B63" s="37" t="n"/>
-      <c r="C63" s="37" t="n"/>
-      <c r="D63" s="43" t="n"/>
-      <c r="E63" s="37" t="n"/>
-      <c r="F63" s="37" t="n"/>
-      <c r="G63" s="37" t="n"/>
-      <c r="H63" s="37" t="n"/>
-      <c r="I63" s="37" t="n"/>
-    </row>
-    <row r="64" ht="15" customHeight="1" s="28">
-      <c r="A64" s="37" t="n"/>
-      <c r="B64" s="37" t="n"/>
-      <c r="C64" s="37" t="n"/>
-      <c r="D64" s="43" t="n"/>
-      <c r="E64" s="37" t="n"/>
-      <c r="F64" s="37" t="n"/>
-      <c r="G64" s="37" t="n"/>
-      <c r="H64" s="37" t="n"/>
-      <c r="I64" s="37" t="n"/>
-    </row>
-    <row r="65" ht="15" customHeight="1" s="28">
-      <c r="A65" s="37" t="n"/>
-      <c r="B65" s="37" t="n"/>
-      <c r="C65" s="37" t="n"/>
-      <c r="D65" s="43" t="n"/>
-      <c r="E65" s="37" t="n"/>
-      <c r="F65" s="37" t="n"/>
-      <c r="G65" s="37" t="n"/>
-      <c r="H65" s="37" t="n"/>
-      <c r="I65" s="37" t="n"/>
-    </row>
-    <row r="66" ht="15" customHeight="1" s="28">
-      <c r="A66" s="37" t="n"/>
-      <c r="B66" s="37" t="n"/>
-      <c r="C66" s="37" t="n"/>
-      <c r="D66" s="43" t="n"/>
-      <c r="E66" s="37" t="n"/>
-      <c r="F66" s="37" t="n"/>
-      <c r="G66" s="37" t="n"/>
-      <c r="H66" s="37" t="n"/>
-      <c r="I66" s="37" t="n"/>
-    </row>
-    <row r="67" ht="15" customHeight="1" s="28">
-      <c r="A67" s="37" t="n"/>
-      <c r="B67" s="37" t="n"/>
-      <c r="C67" s="37" t="n"/>
-      <c r="D67" s="43" t="n"/>
-      <c r="E67" s="37" t="n"/>
-      <c r="F67" s="37" t="n"/>
-      <c r="G67" s="37" t="n"/>
-      <c r="H67" s="37" t="n"/>
-      <c r="I67" s="37" t="n"/>
-    </row>
-    <row r="68" ht="15" customHeight="1" s="28">
-      <c r="A68" s="37" t="n"/>
-      <c r="B68" s="37" t="n"/>
-      <c r="C68" s="37" t="n"/>
-      <c r="D68" s="43" t="n"/>
-      <c r="E68" s="37" t="n"/>
-      <c r="F68" s="37" t="n"/>
-      <c r="G68" s="37" t="n"/>
-      <c r="H68" s="37" t="n"/>
-      <c r="I68" s="37" t="n"/>
-    </row>
-    <row r="69" ht="15" customHeight="1" s="28">
-      <c r="A69" s="37" t="n"/>
-      <c r="B69" s="37" t="n"/>
-      <c r="C69" s="37" t="n"/>
-      <c r="D69" s="43" t="n"/>
-      <c r="E69" s="37" t="n"/>
-      <c r="F69" s="37" t="n"/>
-      <c r="G69" s="37" t="n"/>
-      <c r="H69" s="37" t="n"/>
-      <c r="I69" s="37" t="n"/>
-    </row>
-    <row r="70" ht="15" customHeight="1" s="28">
-      <c r="A70" s="37" t="n"/>
-      <c r="B70" s="37" t="n"/>
-      <c r="C70" s="37" t="n"/>
-      <c r="D70" s="43" t="n"/>
-      <c r="E70" s="37" t="n"/>
-      <c r="F70" s="37" t="n"/>
-      <c r="G70" s="37" t="n"/>
-      <c r="H70" s="37" t="n"/>
-      <c r="I70" s="37" t="n"/>
-    </row>
-    <row r="71" ht="15" customHeight="1" s="28">
-      <c r="A71" s="37" t="n"/>
-      <c r="B71" s="37" t="n"/>
-      <c r="C71" s="37" t="n"/>
-      <c r="D71" s="43" t="n"/>
-      <c r="E71" s="37" t="n"/>
-      <c r="F71" s="37" t="n"/>
-      <c r="G71" s="37" t="n"/>
-      <c r="H71" s="37" t="n"/>
-      <c r="I71" s="37" t="n"/>
-    </row>
-    <row r="72" ht="15" customHeight="1" s="28">
-      <c r="A72" s="37" t="n"/>
-      <c r="B72" s="37" t="n"/>
-      <c r="C72" s="37" t="n"/>
-      <c r="D72" s="43" t="n"/>
-      <c r="E72" s="37" t="n"/>
-      <c r="F72" s="37" t="n"/>
-      <c r="G72" s="37" t="n"/>
-      <c r="H72" s="37" t="n"/>
-      <c r="I72" s="37" t="n"/>
-    </row>
-    <row r="73" ht="15" customHeight="1" s="28">
-      <c r="A73" s="37" t="n"/>
-      <c r="B73" s="37" t="n"/>
-      <c r="C73" s="37" t="n"/>
-      <c r="D73" s="43" t="n"/>
-      <c r="E73" s="37" t="n"/>
-      <c r="F73" s="37" t="n"/>
-      <c r="G73" s="37" t="n"/>
-      <c r="H73" s="37" t="n"/>
-      <c r="I73" s="37" t="n"/>
-    </row>
-    <row r="74" ht="15" customHeight="1" s="28">
-      <c r="A74" s="37" t="n"/>
-      <c r="B74" s="37" t="n"/>
-      <c r="C74" s="37" t="n"/>
-      <c r="D74" s="43" t="n"/>
-      <c r="E74" s="37" t="n"/>
-      <c r="F74" s="37" t="n"/>
-      <c r="G74" s="37" t="n"/>
-      <c r="H74" s="37" t="n"/>
-      <c r="I74" s="37" t="n"/>
-    </row>
-    <row r="75" ht="15" customHeight="1" s="28">
-      <c r="A75" s="37" t="n"/>
-      <c r="B75" s="37" t="n"/>
-      <c r="C75" s="37" t="n"/>
-      <c r="D75" s="43" t="n"/>
-      <c r="E75" s="37" t="n"/>
-      <c r="F75" s="37" t="n"/>
-      <c r="G75" s="37" t="n"/>
-      <c r="H75" s="37" t="n"/>
-      <c r="I75" s="37" t="n"/>
-    </row>
-    <row r="76" ht="15" customHeight="1" s="28">
-      <c r="A76" s="37" t="n"/>
-      <c r="B76" s="37" t="n"/>
-      <c r="C76" s="37" t="n"/>
-      <c r="D76" s="43" t="n"/>
-      <c r="E76" s="37" t="n"/>
-      <c r="F76" s="37" t="n"/>
-      <c r="G76" s="37" t="n"/>
-      <c r="H76" s="37" t="n"/>
-      <c r="I76" s="37" t="n"/>
-    </row>
-    <row r="77" ht="15" customHeight="1" s="28">
-      <c r="A77" s="37" t="n"/>
-      <c r="B77" s="37" t="n"/>
-      <c r="C77" s="37" t="n"/>
-      <c r="D77" s="43" t="n"/>
-      <c r="E77" s="37" t="n"/>
-      <c r="F77" s="37" t="n"/>
-      <c r="G77" s="37" t="n"/>
-      <c r="H77" s="37" t="n"/>
-      <c r="I77" s="37" t="n"/>
-    </row>
-    <row r="78" ht="15" customHeight="1" s="28">
-      <c r="A78" s="37" t="n"/>
-      <c r="B78" s="37" t="n"/>
-      <c r="C78" s="37" t="n"/>
-      <c r="D78" s="43" t="n"/>
-      <c r="E78" s="37" t="n"/>
-      <c r="F78" s="37" t="n"/>
-      <c r="G78" s="37" t="n"/>
-      <c r="H78" s="37" t="n"/>
-      <c r="I78" s="37" t="n"/>
-    </row>
-    <row r="79" ht="15" customHeight="1" s="28">
-      <c r="A79" s="37" t="n"/>
-      <c r="B79" s="37" t="n"/>
-      <c r="C79" s="37" t="n"/>
-      <c r="D79" s="43" t="n"/>
-      <c r="E79" s="37" t="n"/>
-      <c r="F79" s="37" t="n"/>
-      <c r="G79" s="37" t="n"/>
-      <c r="H79" s="37" t="n"/>
-      <c r="I79" s="37" t="n"/>
-    </row>
-    <row r="80" ht="15" customHeight="1" s="28">
-      <c r="A80" s="37" t="n"/>
-      <c r="B80" s="37" t="n"/>
-      <c r="C80" s="37" t="n"/>
-      <c r="D80" s="43" t="n"/>
-      <c r="E80" s="37" t="n"/>
-      <c r="F80" s="37" t="n"/>
-      <c r="G80" s="37" t="n"/>
-      <c r="H80" s="37" t="n"/>
-      <c r="I80" s="37" t="n"/>
-    </row>
-    <row r="81" ht="15" customHeight="1" s="28">
-      <c r="A81" s="37" t="n"/>
-      <c r="B81" s="37" t="n"/>
-      <c r="C81" s="37" t="n"/>
-      <c r="D81" s="43" t="n"/>
-      <c r="E81" s="37" t="n"/>
-      <c r="F81" s="37" t="n"/>
-      <c r="G81" s="37" t="n"/>
-      <c r="H81" s="37" t="n"/>
-      <c r="I81" s="37" t="n"/>
-    </row>
-    <row r="82" ht="15" customHeight="1" s="28">
-      <c r="A82" s="37" t="n"/>
-      <c r="B82" s="37" t="n"/>
-      <c r="C82" s="37" t="n"/>
-      <c r="D82" s="43" t="n"/>
-      <c r="E82" s="37" t="n"/>
-      <c r="F82" s="37" t="n"/>
-      <c r="G82" s="37" t="n"/>
-      <c r="H82" s="37" t="n"/>
-      <c r="I82" s="37" t="n"/>
-    </row>
-    <row r="83" ht="15" customHeight="1" s="28">
-      <c r="A83" s="37" t="n"/>
-      <c r="B83" s="37" t="n"/>
-      <c r="C83" s="37" t="n"/>
-      <c r="D83" s="43" t="n"/>
-      <c r="E83" s="37" t="n"/>
-      <c r="F83" s="37" t="n"/>
-      <c r="G83" s="37" t="n"/>
-      <c r="H83" s="37" t="n"/>
-      <c r="I83" s="37" t="n"/>
-    </row>
-    <row r="84" ht="15" customHeight="1" s="28">
-      <c r="A84" s="37" t="n"/>
-      <c r="B84" s="37" t="n"/>
-      <c r="C84" s="37" t="n"/>
-      <c r="D84" s="43" t="n"/>
-      <c r="E84" s="37" t="n"/>
-      <c r="F84" s="37" t="n"/>
-      <c r="G84" s="37" t="n"/>
-      <c r="H84" s="37" t="n"/>
-      <c r="I84" s="37" t="n"/>
-    </row>
-    <row r="85" ht="15" customHeight="1" s="28">
-      <c r="A85" s="37" t="n"/>
-      <c r="B85" s="37" t="n"/>
-      <c r="C85" s="37" t="n"/>
-      <c r="D85" s="43" t="n"/>
-      <c r="E85" s="37" t="n"/>
-      <c r="F85" s="37" t="n"/>
-      <c r="G85" s="37" t="n"/>
-      <c r="H85" s="37" t="n"/>
-      <c r="I85" s="37" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid BudgetCat" error="Pick from: Housing, Groceries, Utilities, Transport, Childcare, Education…" type="list" errorStyle="stop" operator="between">
-      <formula1>Lists!$K$3:$K$18</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
   <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -7110,7 +5755,7 @@
         <v>8500</v>
       </c>
       <c r="C2" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A2,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A2,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D2" s="43">
@@ -7122,7 +5767,7 @@
         <v/>
       </c>
       <c r="F2" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A2,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A2,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G2" s="37" t="n"/>
@@ -7146,7 +5791,7 @@
         <v>4000</v>
       </c>
       <c r="C3" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A3,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A3,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D3" s="43">
@@ -7158,7 +5803,7 @@
         <v/>
       </c>
       <c r="F3" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A3,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A3,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G3" s="37" t="n"/>
@@ -7173,7 +5818,7 @@
         <v>1500</v>
       </c>
       <c r="C4" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A4,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A4,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D4" s="43">
@@ -7185,7 +5830,7 @@
         <v/>
       </c>
       <c r="F4" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A4,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A4,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G4" s="37" t="n"/>
@@ -7200,7 +5845,7 @@
         <v>5000</v>
       </c>
       <c r="C5" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A5,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A5,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D5" s="43">
@@ -7212,7 +5857,7 @@
         <v/>
       </c>
       <c r="F5" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A5,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A5,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G5" s="37" t="n"/>
@@ -7227,7 +5872,7 @@
         <v>1200</v>
       </c>
       <c r="C6" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A6,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A6,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D6" s="43">
@@ -7239,7 +5884,7 @@
         <v/>
       </c>
       <c r="F6" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A6,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A6,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G6" s="37" t="n"/>
@@ -7254,7 +5899,7 @@
         <v>800</v>
       </c>
       <c r="C7" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A7,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A7,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D7" s="43">
@@ -7266,7 +5911,7 @@
         <v/>
       </c>
       <c r="F7" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A7,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A7,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G7" s="37" t="n"/>
@@ -7281,7 +5926,7 @@
         <v>800</v>
       </c>
       <c r="C8" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A8,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A8,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D8" s="43">
@@ -7293,7 +5938,7 @@
         <v/>
       </c>
       <c r="F8" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A8,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A8,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G8" s="37" t="n"/>
@@ -7308,7 +5953,7 @@
         <v>1000</v>
       </c>
       <c r="C9" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A9,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A9,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D9" s="43">
@@ -7320,7 +5965,7 @@
         <v/>
       </c>
       <c r="F9" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A9,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A9,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G9" s="37" t="n"/>
@@ -7335,7 +5980,7 @@
         <v>400</v>
       </c>
       <c r="C10" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A10,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A10,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D10" s="43">
@@ -7347,7 +5992,7 @@
         <v/>
       </c>
       <c r="F10" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A10,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A10,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G10" s="37" t="n"/>
@@ -7362,7 +6007,7 @@
         <v>5000</v>
       </c>
       <c r="C11" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A11,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A11,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D11" s="43">
@@ -7374,7 +6019,7 @@
         <v/>
       </c>
       <c r="F11" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A11,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A11,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G11" s="37" t="n"/>
@@ -7389,7 +6034,7 @@
         <v>500</v>
       </c>
       <c r="C12" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A12,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Txns'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A12,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
         <v/>
       </c>
       <c r="D12" s="43">
@@ -7401,7 +6046,7 @@
         <v/>
       </c>
       <c r="F12" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Txns'!D:D,'Finance-Txns'!E:E,A12,'Finance-Txns'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Txns'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A12,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
         <v/>
       </c>
       <c r="G12" s="37" t="n"/>
@@ -7448,7 +6093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7758,4 +6403,377 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="12" customWidth="1" style="27" min="1" max="1"/>
+    <col width="22" customWidth="1" style="27" min="2" max="2"/>
+    <col width="16" customWidth="1" style="27" min="3" max="3"/>
+    <col width="18" customWidth="1" style="27" min="4" max="4"/>
+    <col width="14" customWidth="1" style="27" min="5" max="5"/>
+    <col width="18" customWidth="1" style="27" min="6" max="6"/>
+    <col width="28" customWidth="1" style="27" min="7" max="8"/>
+    <col width="24" customWidth="1" style="27" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1" s="28">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Child</t>
+        </is>
+      </c>
+      <c r="B1" s="34" t="inlineStr">
+        <is>
+          <t>Institution</t>
+        </is>
+      </c>
+      <c r="C1" s="34" t="inlineStr">
+        <is>
+          <t>Year/Grade</t>
+        </is>
+      </c>
+      <c r="D1" s="34" t="inlineStr">
+        <is>
+          <t>Teacher/Caregiver</t>
+        </is>
+      </c>
+      <c r="E1" s="34" t="inlineStr">
+        <is>
+          <t>Next Key Date</t>
+        </is>
+      </c>
+      <c r="F1" s="34" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" s="34" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="H1" s="34" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="I1" s="34" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1" s="28">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>[Child 1]</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>[Preschool name]</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>Gan Trom-Hova</t>
+        </is>
+      </c>
+      <c r="D2" s="35" t="inlineStr">
+        <is>
+          <t>[Teacher]</t>
+        </is>
+      </c>
+      <c r="E2" s="36" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F2" s="35" t="inlineStr">
+        <is>
+          <t>School year start</t>
+        </is>
+      </c>
+      <c r="G2" s="35" t="inlineStr">
+        <is>
+          <t>Buy supplies, label clothes</t>
+        </is>
+      </c>
+      <c r="H2" s="35" t="inlineStr">
+        <is>
+          <t>[teacher@school]</t>
+        </is>
+      </c>
+      <c r="I2" s="35" t="n"/>
+    </row>
+    <row r="3" ht="36" customHeight="1" s="28">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>[Child 1]</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>[Preschool name]</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Gan Trom-Hova</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>[Teacher]</t>
+        </is>
+      </c>
+      <c r="E3" s="36" t="n">
+        <v>46346</v>
+      </c>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>Parent-teacher</t>
+        </is>
+      </c>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Schedule meeting slot</t>
+        </is>
+      </c>
+      <c r="H3" s="35" t="inlineStr">
+        <is>
+          <t>[teacher@school]</t>
+        </is>
+      </c>
+      <c r="I3" s="35" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1" s="28">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>[Child 2]</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>[Daycare name]</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Maon</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>[Caregiver]</t>
+        </is>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>46371</v>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>1st-grade registration opens</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Register on city portal</t>
+        </is>
+      </c>
+      <c r="H4" s="35" t="inlineStr">
+        <is>
+          <t>[city helpdesk]</t>
+        </is>
+      </c>
+      <c r="I4" s="35" t="inlineStr">
+        <is>
+          <t>Adar to lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="28">
+      <c r="A5" s="37" t="n"/>
+      <c r="B5" s="37" t="n"/>
+      <c r="C5" s="37" t="n"/>
+      <c r="D5" s="37" t="n"/>
+      <c r="E5" s="37" t="n"/>
+      <c r="F5" s="37" t="n"/>
+      <c r="G5" s="37" t="n"/>
+      <c r="H5" s="37" t="n"/>
+      <c r="I5" s="37" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="28">
+      <c r="A6" s="37" t="n"/>
+      <c r="B6" s="37" t="n"/>
+      <c r="C6" s="37" t="n"/>
+      <c r="D6" s="37" t="n"/>
+      <c r="E6" s="37" t="n"/>
+      <c r="F6" s="37" t="n"/>
+      <c r="G6" s="37" t="n"/>
+      <c r="H6" s="37" t="n"/>
+      <c r="I6" s="37" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="28">
+      <c r="A7" s="37" t="n"/>
+      <c r="B7" s="37" t="n"/>
+      <c r="C7" s="37" t="n"/>
+      <c r="D7" s="37" t="n"/>
+      <c r="E7" s="37" t="n"/>
+      <c r="F7" s="37" t="n"/>
+      <c r="G7" s="37" t="n"/>
+      <c r="H7" s="37" t="n"/>
+      <c r="I7" s="37" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="28">
+      <c r="A8" s="37" t="n"/>
+      <c r="B8" s="37" t="n"/>
+      <c r="C8" s="37" t="n"/>
+      <c r="D8" s="37" t="n"/>
+      <c r="E8" s="37" t="n"/>
+      <c r="F8" s="37" t="n"/>
+      <c r="G8" s="37" t="n"/>
+      <c r="H8" s="37" t="n"/>
+      <c r="I8" s="37" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="28">
+      <c r="A9" s="37" t="n"/>
+      <c r="B9" s="37" t="n"/>
+      <c r="C9" s="37" t="n"/>
+      <c r="D9" s="37" t="n"/>
+      <c r="E9" s="37" t="n"/>
+      <c r="F9" s="37" t="n"/>
+      <c r="G9" s="37" t="n"/>
+      <c r="H9" s="37" t="n"/>
+      <c r="I9" s="37" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="28">
+      <c r="A10" s="37" t="n"/>
+      <c r="B10" s="37" t="n"/>
+      <c r="C10" s="37" t="n"/>
+      <c r="D10" s="37" t="n"/>
+      <c r="E10" s="37" t="n"/>
+      <c r="F10" s="37" t="n"/>
+      <c r="G10" s="37" t="n"/>
+      <c r="H10" s="37" t="n"/>
+      <c r="I10" s="37" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="28">
+      <c r="A11" s="37" t="n"/>
+      <c r="B11" s="37" t="n"/>
+      <c r="C11" s="37" t="n"/>
+      <c r="D11" s="37" t="n"/>
+      <c r="E11" s="37" t="n"/>
+      <c r="F11" s="37" t="n"/>
+      <c r="G11" s="37" t="n"/>
+      <c r="H11" s="37" t="n"/>
+      <c r="I11" s="37" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="28">
+      <c r="A12" s="37" t="n"/>
+      <c r="B12" s="37" t="n"/>
+      <c r="C12" s="37" t="n"/>
+      <c r="D12" s="37" t="n"/>
+      <c r="E12" s="37" t="n"/>
+      <c r="F12" s="37" t="n"/>
+      <c r="G12" s="37" t="n"/>
+      <c r="H12" s="37" t="n"/>
+      <c r="I12" s="37" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="28">
+      <c r="A13" s="37" t="n"/>
+      <c r="B13" s="37" t="n"/>
+      <c r="C13" s="37" t="n"/>
+      <c r="D13" s="37" t="n"/>
+      <c r="E13" s="37" t="n"/>
+      <c r="F13" s="37" t="n"/>
+      <c r="G13" s="37" t="n"/>
+      <c r="H13" s="37" t="n"/>
+      <c r="I13" s="37" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="28">
+      <c r="A14" s="37" t="n"/>
+      <c r="B14" s="37" t="n"/>
+      <c r="C14" s="37" t="n"/>
+      <c r="D14" s="37" t="n"/>
+      <c r="E14" s="37" t="n"/>
+      <c r="F14" s="37" t="n"/>
+      <c r="G14" s="37" t="n"/>
+      <c r="H14" s="37" t="n"/>
+      <c r="I14" s="37" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="28">
+      <c r="A15" s="37" t="n"/>
+      <c r="B15" s="37" t="n"/>
+      <c r="C15" s="37" t="n"/>
+      <c r="D15" s="37" t="n"/>
+      <c r="E15" s="37" t="n"/>
+      <c r="F15" s="37" t="n"/>
+      <c r="G15" s="37" t="n"/>
+      <c r="H15" s="37" t="n"/>
+      <c r="I15" s="37" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="28">
+      <c r="A16" s="37" t="n"/>
+      <c r="B16" s="37" t="n"/>
+      <c r="C16" s="37" t="n"/>
+      <c r="D16" s="37" t="n"/>
+      <c r="E16" s="37" t="n"/>
+      <c r="F16" s="37" t="n"/>
+      <c r="G16" s="37" t="n"/>
+      <c r="H16" s="37" t="n"/>
+      <c r="I16" s="37" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="28">
+      <c r="A17" s="37" t="n"/>
+      <c r="B17" s="37" t="n"/>
+      <c r="C17" s="37" t="n"/>
+      <c r="D17" s="37" t="n"/>
+      <c r="E17" s="37" t="n"/>
+      <c r="F17" s="37" t="n"/>
+      <c r="G17" s="37" t="n"/>
+      <c r="H17" s="37" t="n"/>
+      <c r="I17" s="37" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="28">
+      <c r="A18" s="37" t="n"/>
+      <c r="B18" s="37" t="n"/>
+      <c r="C18" s="37" t="n"/>
+      <c r="D18" s="37" t="n"/>
+      <c r="E18" s="37" t="n"/>
+      <c r="F18" s="37" t="n"/>
+      <c r="G18" s="37" t="n"/>
+      <c r="H18" s="37" t="n"/>
+      <c r="I18" s="37" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="28">
+      <c r="A19" s="37" t="n"/>
+      <c r="B19" s="37" t="n"/>
+      <c r="C19" s="37" t="n"/>
+      <c r="D19" s="37" t="n"/>
+      <c r="E19" s="37" t="n"/>
+      <c r="F19" s="37" t="n"/>
+      <c r="G19" s="37" t="n"/>
+      <c r="H19" s="37" t="n"/>
+      <c r="I19" s="37" t="n"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E1000">
+    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="4" text="" percent="0" bottom="0">
+      <formula>AND(ISNUMBER(E2),E2&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="0" text="" percent="0" bottom="0">
+      <formula>AND(ISNUMBER(E2),E2-TODAY()&gt;=0,E2-TODAY()&lt;=30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
M6.4: finance categorizer + budget reconciliation (D-050/051)
On-box rules engine (categorize.py + committed, non-personal 14_Finance_Category_Rules.csv) fills Category/Cat-Source at ingest; DeepSeek gap-fills the rules-miss remainder (description + amount only, SPEC 8.6). Reconciliation: Finance-Budget actuals move from a serial DATE() SUMIFS (read 0 vs the RAW ISO-text Date) to a locale-independent text-prefix wildcard, chosen over USER_ENTERED append (would coerce Txn-ID/Account and break dedup); append stays RAW. Added Last Month (ILS) column for MoM; briefing Money section gained per-category + MoM. Seed formulas updated + pinned by a test. PROVISIONAL vocab until Shanee's budget migration.
</commit_message>
<xml_diff>
--- a/Family_OS.xlsx
+++ b/Family_OS.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendars" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar-Events" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reminders" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance-Accounts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance-Budget" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goals" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Education" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Car" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="14" state="hidden" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhatsApp_Inbox" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhatsApp_Archive" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance-Transactions" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="People" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Calendars" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Calendar-Events" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reminders" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Finance-Accounts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Finance-Budget" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Goals" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Education" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Health" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Car" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Contacts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Contracts" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Lists" sheetId="14" state="hidden" r:id="rId14"/>
+    <sheet name="Settings" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="WhatsApp_Inbox" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="WhatsApp_Archive" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finance-Transactions" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -3331,122 +3331,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>Amount (ILS)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="27" t="inlineStr">
         <is>
           <t>Cat-Source</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="27" t="inlineStr">
         <is>
           <t>Txn-ID</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="27" t="inlineStr">
         <is>
           <t>Imported-At</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>[Joint Checking]</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>SHUFERSAL DEAL</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="27" t="n">
         <v>-432.5</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>Groceries</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>sample</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="27" t="inlineStr">
         <is>
           <t>sample-1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="27" t="inlineStr">
         <is>
           <t>2026-05-11T06:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>[Visa Cal — Adar]</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
         <is>
           <t>PAZ GAS STATION</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="27" t="n">
         <v>-280</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="27" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="27" t="inlineStr">
         <is>
           <t>sample</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="27" t="inlineStr">
         <is>
           <t>sample-2</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="27" t="inlineStr">
         <is>
           <t>2026-05-11T06:00:00</t>
         </is>
@@ -5689,7 +5689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="27" min="1" max="3"/>
@@ -5744,6 +5744,11 @@
         <f>TODAY()</f>
         <v/>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Last Month (ILS)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="28">
       <c r="A2" s="37" t="inlineStr">
@@ -5755,7 +5760,7 @@
         <v>8500</v>
       </c>
       <c r="C2" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A2,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A2,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D2" s="43">
@@ -5767,7 +5772,7 @@
         <v/>
       </c>
       <c r="F2" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A2,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A2,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G2" s="37" t="n"/>
@@ -5780,6 +5785,10 @@
         <f>TEXT(I1,"yyyy-mm")</f>
         <v/>
       </c>
+      <c r="J2">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A2,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="37" t="inlineStr">
@@ -5791,7 +5800,7 @@
         <v>4000</v>
       </c>
       <c r="C3" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A3,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A3,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D3" s="43">
@@ -5803,10 +5812,23 @@
         <v/>
       </c>
       <c r="F3" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A3,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A3,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G3" s="37" t="n"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Prev month tag</t>
+        </is>
+      </c>
+      <c r="I3">
+        <f>TEXT(EDATE($I$1,-1),"yyyy-mm")</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A3,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="28">
       <c r="A4" s="37" t="inlineStr">
@@ -5818,7 +5840,7 @@
         <v>1500</v>
       </c>
       <c r="C4" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A4,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A4,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D4" s="43">
@@ -5830,10 +5852,14 @@
         <v/>
       </c>
       <c r="F4" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A4,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A4,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G4" s="37" t="n"/>
+      <c r="J4">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A4,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="28">
       <c r="A5" s="37" t="inlineStr">
@@ -5845,7 +5871,7 @@
         <v>5000</v>
       </c>
       <c r="C5" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A5,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A5,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D5" s="43">
@@ -5857,10 +5883,14 @@
         <v/>
       </c>
       <c r="F5" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A5,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A5,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G5" s="37" t="n"/>
+      <c r="J5">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A5,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="28">
       <c r="A6" s="37" t="inlineStr">
@@ -5872,7 +5902,7 @@
         <v>1200</v>
       </c>
       <c r="C6" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A6,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A6,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D6" s="43">
@@ -5884,10 +5914,14 @@
         <v/>
       </c>
       <c r="F6" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A6,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A6,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G6" s="37" t="n"/>
+      <c r="J6">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A6,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="28">
       <c r="A7" s="37" t="inlineStr">
@@ -5899,7 +5933,7 @@
         <v>800</v>
       </c>
       <c r="C7" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A7,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A7,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D7" s="43">
@@ -5911,10 +5945,14 @@
         <v/>
       </c>
       <c r="F7" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A7,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A7,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G7" s="37" t="n"/>
+      <c r="J7">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A7,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="28">
       <c r="A8" s="37" t="inlineStr">
@@ -5926,7 +5964,7 @@
         <v>800</v>
       </c>
       <c r="C8" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A8,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A8,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D8" s="43">
@@ -5938,10 +5976,14 @@
         <v/>
       </c>
       <c r="F8" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A8,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A8,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G8" s="37" t="n"/>
+      <c r="J8">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A8,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="28">
       <c r="A9" s="37" t="inlineStr">
@@ -5953,7 +5995,7 @@
         <v>1000</v>
       </c>
       <c r="C9" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A9,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A9,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D9" s="43">
@@ -5965,10 +6007,14 @@
         <v/>
       </c>
       <c r="F9" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A9,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A9,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G9" s="37" t="n"/>
+      <c r="J9">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A9,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="28">
       <c r="A10" s="37" t="inlineStr">
@@ -5980,7 +6026,7 @@
         <v>400</v>
       </c>
       <c r="C10" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A10,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A10,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D10" s="43">
@@ -5992,10 +6038,14 @@
         <v/>
       </c>
       <c r="F10" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A10,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A10,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G10" s="37" t="n"/>
+      <c r="J10">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A10,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="28">
       <c r="A11" s="37" t="inlineStr">
@@ -6007,7 +6057,7 @@
         <v>5000</v>
       </c>
       <c r="C11" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A11,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A11,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D11" s="43">
@@ -6019,10 +6069,14 @@
         <v/>
       </c>
       <c r="F11" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A11,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A11,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G11" s="37" t="n"/>
+      <c r="J11">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A11,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="28">
       <c r="A12" s="37" t="inlineStr">
@@ -6034,7 +6088,7 @@
         <v>500</v>
       </c>
       <c r="C12" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A12,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),MONTH($I$1),1),'Finance-Transactions'!A:A,"&lt;"&amp;DATE(YEAR($I$1),MONTH($I$1)+1,1)),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A12,'Finance-Transactions'!A:A,$I$2&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="D12" s="43">
@@ -6046,10 +6100,14 @@
         <v/>
       </c>
       <c r="F12" s="43">
-        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,A12,'Finance-Transactions'!A:A,"&gt;="&amp;DATE(YEAR($I$1),1,1),'Finance-Transactions'!A:A,"&lt;="&amp;$I$1),0)</f>
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A12,'Finance-Transactions'!A:A,TEXT($I$1,"yyyy")&amp;"*"),0)</f>
         <v/>
       </c>
       <c r="G12" s="37" t="n"/>
+      <c r="J12">
+        <f>IFERROR(-SUMIFS('Finance-Transactions'!D:D,'Finance-Transactions'!E:E,$A12,'Finance-Transactions'!A:A,$I$3&amp;"*"),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="28">
       <c r="A13" s="48" t="inlineStr">

</xml_diff>